<commit_message>
fase 1 se agregan ultimos datos
</commit_message>
<xml_diff>
--- a/COLABORADORES.xlsx
+++ b/COLABORADORES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Developer user\android\williApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC506153-721F-4315-9E6B-BF28725F53F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D6B1C97-AF58-497B-BF2D-BC417543AA27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{514F16AA-81CC-4F51-8586-9ACBD73BDCD3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{514F16AA-81CC-4F51-8586-9ACBD73BDCD3}"/>
   </bookViews>
   <sheets>
     <sheet name="Colaboradores" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Equipos" sheetId="4" r:id="rId3"/>
     <sheet name="TipoMantenimiento" sheetId="5" r:id="rId4"/>
     <sheet name="LugaresMantenimiento" sheetId="6" r:id="rId5"/>
-    <sheet name="TecnicosManteniemiento" sheetId="7" r:id="rId6"/>
+    <sheet name="Operadores y supervisores" sheetId="7" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="124">
   <si>
     <t>Colaboradores</t>
   </si>
@@ -218,18 +218,9 @@
     <t xml:space="preserve">Planta Clemencia </t>
   </si>
   <si>
-    <t>Num Tecnicos Mantenimientos</t>
-  </si>
-  <si>
-    <t>Eider Meléndez</t>
-  </si>
-  <si>
     <t>Gualberto Albor</t>
   </si>
   <si>
-    <t>Wilfredo Ramirez</t>
-  </si>
-  <si>
     <t>TECNICOS</t>
   </si>
   <si>
@@ -399,6 +390,18 @@
   </si>
   <si>
     <t>EXCAVADORA</t>
+  </si>
+  <si>
+    <t>Eider Melendez</t>
+  </si>
+  <si>
+    <t>José Julián de la Ossa</t>
+  </si>
+  <si>
+    <t>Ismendy Ruiz</t>
+  </si>
+  <si>
+    <t>Num de Tecnicos</t>
   </si>
 </sst>
 </file>
@@ -492,7 +495,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -525,7 +528,6 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -844,14 +846,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A57C91-D5F8-43D7-BBC5-0072E1A875CB}">
   <dimension ref="A1:D64"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.44140625" customWidth="1"/>
-    <col min="2" max="2" width="32.6640625" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -860,7 +862,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>48</v>
       </c>
@@ -871,7 +873,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>1</v>
       </c>
@@ -880,7 +882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -891,7 +893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -902,7 +904,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
@@ -913,7 +915,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -924,7 +926,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>28</v>
       </c>
@@ -932,11 +934,11 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
     </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>1</v>
       </c>
@@ -945,7 +947,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>2</v>
       </c>
@@ -956,7 +958,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>3</v>
       </c>
@@ -967,7 +969,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>4</v>
       </c>
@@ -978,7 +980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
@@ -989,7 +991,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>28</v>
       </c>
@@ -1000,32 +1002,32 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
-      <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D16" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B17" s="13"/>
       <c r="D17" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>3</v>
       </c>
@@ -1033,7 +1035,7 @@
         <v>8604171</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>4</v>
       </c>
@@ -1041,7 +1043,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>5</v>
       </c>
@@ -1049,7 +1051,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>28</v>
       </c>
@@ -1057,17 +1059,17 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
     </row>
-    <row r="24" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B24" s="13"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>2</v>
       </c>
@@ -1075,7 +1077,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>3</v>
       </c>
@@ -1083,7 +1085,7 @@
         <v>1063277243</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>4</v>
       </c>
@@ -1091,7 +1093,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>5</v>
       </c>
@@ -1099,7 +1101,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>28</v>
       </c>
@@ -1107,17 +1109,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
     </row>
-    <row r="31" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B31" s="13"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>2</v>
       </c>
@@ -1125,7 +1127,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>3</v>
       </c>
@@ -1133,7 +1135,7 @@
         <v>3738908</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>4</v>
       </c>
@@ -1141,7 +1143,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>5</v>
       </c>
@@ -1149,7 +1151,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>28</v>
       </c>
@@ -1157,17 +1159,17 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
     </row>
-    <row r="38" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B38" s="13"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>2</v>
       </c>
@@ -1175,7 +1177,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>3</v>
       </c>
@@ -1183,7 +1185,7 @@
         <v>1047438805</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>4</v>
       </c>
@@ -1191,7 +1193,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>5</v>
       </c>
@@ -1199,7 +1201,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>28</v>
       </c>
@@ -1207,17 +1209,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
     </row>
-    <row r="45" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B45" s="13"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>2</v>
       </c>
@@ -1225,7 +1227,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>3</v>
       </c>
@@ -1233,7 +1235,7 @@
         <v>1050200236</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>4</v>
       </c>
@@ -1241,7 +1243,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>5</v>
       </c>
@@ -1249,7 +1251,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>28</v>
       </c>
@@ -1257,17 +1259,17 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
       <c r="B51" s="7"/>
     </row>
-    <row r="52" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B52" s="13"/>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>2</v>
       </c>
@@ -1275,7 +1277,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>3</v>
       </c>
@@ -1283,7 +1285,7 @@
         <v>5820371</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>4</v>
       </c>
@@ -1291,7 +1293,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>5</v>
       </c>
@@ -1299,7 +1301,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>28</v>
       </c>
@@ -1307,17 +1309,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
       <c r="B58" s="7"/>
     </row>
-    <row r="59" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B59" s="13"/>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>2</v>
       </c>
@@ -1325,7 +1327,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>3</v>
       </c>
@@ -1333,7 +1335,7 @@
         <v>80110706</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>4</v>
       </c>
@@ -1341,7 +1343,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>5</v>
       </c>
@@ -1349,7 +1351,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>28</v>
       </c>
@@ -1374,7 +1376,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6 B13 B20 B27 B34 B41 B48 B55 B62" xr:uid="{92097CCC-FDD3-4076-BD23-15E3B0D70A81}">
       <formula1>$D$2:$D$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7 B14 B21 B63 B35 B42 B49 B56 B28" xr:uid="{42457374-A317-4DF1-B09F-CD3E63FEBB13}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7 B14 B21 B63 B35 B42 B49 B56 B28 D16" xr:uid="{42457374-A317-4DF1-B09F-CD3E63FEBB13}">
       <formula1>$D$11:$D$18</formula1>
     </dataValidation>
   </dataValidations>
@@ -1385,19 +1387,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25EDE15-20FC-4616-A1B6-6A14C549E38C}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.44140625" customWidth="1"/>
-    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>44</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>43</v>
       </c>
@@ -1405,13 +1407,13 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>45</v>
       </c>
       <c r="B3" s="13"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1419,7 +1421,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
@@ -1427,7 +1429,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
@@ -1435,7 +1437,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>4</v>
       </c>
@@ -1443,7 +1445,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>5</v>
       </c>
@@ -1463,662 +1465,662 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DEFEEF3-00B0-4CA4-9DF7-AFF732E96F7D}">
   <dimension ref="A1:E89"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.21875" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>46</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B2" s="10">
         <v>8</v>
       </c>
-      <c r="D2" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="E2" s="15"/>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="D2" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="E2" s="14"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B3" s="13"/>
       <c r="D3" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E3" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E4" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E5" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B10" s="5"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B11" s="14">
+        <v>117</v>
+      </c>
+      <c r="B11" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
     </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="13"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B14" s="13"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="6" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B21" s="5"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B22" s="14">
+        <v>117</v>
+      </c>
+      <c r="B22" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="13"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" s="13"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B26" s="6" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B30" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="B31" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B32" s="5"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B33" s="14">
+        <v>117</v>
+      </c>
+      <c r="B33" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="13"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B36" s="13"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B37" s="6" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" s="6" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B41" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="B42" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B43" s="5"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B44" s="14">
+        <v>117</v>
+      </c>
+      <c r="B44" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B45" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B47" s="13"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B47" s="13"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B48" s="6" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="5" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B52" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="B53" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B54" s="5"/>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B55" s="14">
+        <v>117</v>
+      </c>
+      <c r="B55" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B56" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B58" s="13"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B60" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B58" s="13"/>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B59" s="6" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="5" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B62" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="5" t="s">
-        <v>111</v>
-      </c>
       <c r="B65" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B66" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+      <c r="B66" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B69" s="13"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B71" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="5" t="s">
+      <c r="B74" s="5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B72" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B73" s="6" t="s">
+      <c r="B75" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B77" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B77" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B80" s="13"/>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B82" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A83" s="5" t="s">
+      <c r="B85" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B83" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A84" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B84" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A85" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A86" s="5" t="s">
-        <v>73</v>
-      </c>
       <c r="B86" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B87" s="5"/>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B88" s="14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+      <c r="B88" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2141,19 +2143,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FA027EA-D30C-4F34-AE5B-C885EFD4874C}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.88671875" customWidth="1"/>
-    <col min="2" max="2" width="21.88671875" customWidth="1"/>
+    <col min="1" max="1" width="29.85546875" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>57</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>49</v>
       </c>
@@ -2161,13 +2163,13 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="13"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -2175,7 +2177,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
@@ -2183,7 +2185,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
@@ -2191,7 +2193,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>4</v>
       </c>
@@ -2199,7 +2201,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>5</v>
       </c>
@@ -2207,7 +2209,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>6</v>
       </c>
@@ -2227,19 +2229,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3760A244-362C-4EF9-A5E8-570E9E41365B}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.21875" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>58</v>
       </c>
@@ -2247,13 +2249,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="13"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -2261,7 +2263,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
@@ -2269,7 +2271,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
@@ -2288,55 +2290,63 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EAD5EC-7102-411B-AF6C-419F874E24FA}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.109375" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>62</v>
+        <v>123</v>
       </c>
       <c r="B2" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>56</v>
       </c>
       <c r="B3" s="13"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>1</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>65</v>
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>